<commit_message>
Updated PERT Sheet to replace older version
Added two new columns
</commit_message>
<xml_diff>
--- a/Plan/PERT Sheet .xlsx
+++ b/Plan/PERT Sheet .xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stuartbaker/Desktop/University/Year2/Software Engineering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C2E3D2C-F37D-5646-AABB-864485E6D9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{93F180D2-BFA7-8C40-9E82-DC8D50C842ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{409E12EB-2986-7040-875A-ECA154068229}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="95">
   <si>
     <t>Task</t>
   </si>
@@ -288,6 +288,39 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Ontime Completion?</t>
+  </si>
+  <si>
+    <t>Yes, day 3</t>
+  </si>
+  <si>
+    <t>Yes, day 6</t>
+  </si>
+  <si>
+    <t>Yes, day 9</t>
+  </si>
+  <si>
+    <t>Yes, day 12</t>
+  </si>
+  <si>
+    <t>Misinterpretation and ambiguity in the specification led to questions being raised to Mr Raffles for clarity</t>
+  </si>
+  <si>
+    <t>Setbacks and Reasons</t>
+  </si>
+  <si>
+    <t>Yes, day 15</t>
+  </si>
+  <si>
+    <t>Took longer than planned due to illness and misreading the brief. At first we thought we designed our own board, but then we realised there was an excel sheet stating the different tile properties</t>
+  </si>
+  <si>
+    <t>Yes, day 16</t>
+  </si>
+  <si>
+    <t>Later start for this as we were focussed on other aspects of the game. This was not a priority at the time and also wasn't part of the critical path so we had some slack time.</t>
   </si>
 </sst>
 </file>
@@ -368,7 +401,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -377,19 +410,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -724,21 +755,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{904A3F7C-A719-FE4F-BE6A-42977A5F0A83}">
-  <dimension ref="B2:J23"/>
+  <dimension ref="B2:L23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="82.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="20" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:12" ht="20" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -766,15 +799,21 @@
       <c r="J2" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="3" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K2" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="3">
         <v>3</v>
       </c>
       <c r="E3" s="3" t="s">
@@ -792,18 +831,22 @@
       <c r="I3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="4" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K3" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="4">
         <v>3</v>
       </c>
       <c r="E4" s="4" t="s">
@@ -821,18 +864,22 @@
       <c r="I4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="6" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="5" spans="2:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="L4" s="4"/>
+    </row>
+    <row r="5" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>3</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -850,18 +897,22 @@
       <c r="I5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="6" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K5" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="4">
         <v>3</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -879,18 +930,22 @@
       <c r="I6" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="6" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="7" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L6" s="4"/>
+    </row>
+    <row r="7" spans="2:12" ht="34" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="3">
         <v>3</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -908,18 +963,24 @@
       <c r="I7" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="8" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K7" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="4">
         <v>3</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -937,18 +998,22 @@
       <c r="I8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="6" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="9" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K8" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="L8" s="4"/>
+    </row>
+    <row r="9" spans="2:12" ht="34" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>3</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -966,18 +1031,24 @@
       <c r="I9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="10" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K9" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="34" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="4">
         <v>3</v>
       </c>
       <c r="E10" s="4" t="s">
@@ -995,18 +1066,24 @@
       <c r="I10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="6" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="11" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K10" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>3</v>
       </c>
       <c r="E11" s="3" t="s">
@@ -1024,18 +1101,22 @@
       <c r="I11" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="12" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K11" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="4">
         <v>36</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -1053,18 +1134,20 @@
       <c r="I12" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="6" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="13" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K12" s="6"/>
+      <c r="L12" s="4"/>
+    </row>
+    <row r="13" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>24</v>
       </c>
       <c r="E13" s="3" t="s">
@@ -1082,18 +1165,20 @@
       <c r="I13" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="14" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K13" s="5"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="4">
         <v>24</v>
       </c>
       <c r="E14" s="4" t="s">
@@ -1111,18 +1196,20 @@
       <c r="I14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="6" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="15" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K14" s="6"/>
+      <c r="L14" s="4"/>
+    </row>
+    <row r="15" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="3">
         <v>24</v>
       </c>
       <c r="E15" s="3" t="s">
@@ -1140,18 +1227,20 @@
       <c r="I15" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="J15" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="16" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K15" s="5"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B16" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="4">
         <v>36</v>
       </c>
       <c r="E16" s="4" t="s">
@@ -1169,18 +1258,20 @@
       <c r="I16" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="6" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="17" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K16" s="6"/>
+      <c r="L16" s="4"/>
+    </row>
+    <row r="17" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B17" s="3" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="3">
         <v>6</v>
       </c>
       <c r="E17" s="3" t="s">
@@ -1198,18 +1289,20 @@
       <c r="I17" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="18" spans="2:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K17" s="5"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="4">
         <v>42</v>
       </c>
       <c r="E18" s="4" t="s">
@@ -1227,18 +1320,20 @@
       <c r="I18" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="6" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="19" spans="2:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K18" s="6"/>
+      <c r="L18" s="4"/>
+    </row>
+    <row r="19" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="3">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="s">
@@ -1256,18 +1351,20 @@
       <c r="I19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="J19" s="6" t="s">
+      <c r="J19" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="20" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K19" s="5"/>
+      <c r="L19" s="3"/>
+    </row>
+    <row r="20" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B20" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="4">
         <v>6</v>
       </c>
       <c r="E20" s="4" t="s">
@@ -1285,18 +1382,20 @@
       <c r="I20" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="J20" s="6" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="21" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K20" s="6"/>
+      <c r="L20" s="4"/>
+    </row>
+    <row r="21" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="3">
         <v>3</v>
       </c>
       <c r="E21" s="3" t="s">
@@ -1314,18 +1413,20 @@
       <c r="I21" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="J21" s="6" t="s">
+      <c r="J21" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="22" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K21" s="5"/>
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="4">
         <v>3</v>
       </c>
       <c r="E22" s="4" t="s">
@@ -1343,18 +1444,20 @@
       <c r="I22" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="J22" s="6" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="23" spans="2:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="K22" s="6"/>
+      <c r="L22" s="4"/>
+    </row>
+    <row r="23" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B23" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="3">
         <v>0</v>
       </c>
       <c r="E23" s="3" t="s">
@@ -1372,9 +1475,11 @@
       <c r="I23" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J23" s="6" t="s">
+      <c r="J23" s="5" t="s">
         <v>82</v>
       </c>
+      <c r="K23" s="5"/>
+      <c r="L23" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>